<commit_message>
chore: regenerate vocabulary workbook from schema
</commit_message>
<xml_diff>
--- a/docs/assets/coremeta4cat_vocabulary.xlsx
+++ b/docs/assets/coremeta4cat_vocabulary.xlsx
@@ -2797,7 +2797,7 @@
       <c r="H37" s="12" t="inlineStr"/>
       <c r="I37" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J37" s="12" t="inlineStr">
@@ -3883,7 +3883,7 @@
       <c r="H64" s="12" t="inlineStr"/>
       <c r="I64" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J64" s="12" t="inlineStr">
@@ -7077,7 +7077,7 @@
       <c r="H138" s="12" t="inlineStr"/>
       <c r="I138" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J138" s="12" t="inlineStr">
@@ -7992,7 +7992,7 @@
       <c r="H159" s="12" t="inlineStr"/>
       <c r="I159" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J159" s="12" t="inlineStr">
@@ -10482,7 +10482,7 @@
       <c r="H216" s="12" t="inlineStr"/>
       <c r="I216" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J216" s="12" t="inlineStr">
@@ -16020,7 +16020,7 @@
       <c r="H131" s="12" t="inlineStr"/>
       <c r="I131" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J131" s="12" t="inlineStr">
@@ -16302,7 +16302,7 @@
       <c r="H138" s="12" t="inlineStr"/>
       <c r="I138" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J138" s="12" t="inlineStr">
@@ -16511,7 +16511,7 @@
       <c r="H143" s="12" t="inlineStr"/>
       <c r="I143" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J143" s="12" t="inlineStr">
@@ -20589,7 +20589,7 @@
       <c r="H238" s="12" t="inlineStr"/>
       <c r="I238" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:heating_ramp</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J238" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Add CatalystTypes & PerformanceMeasures
</commit_message>
<xml_diff>
--- a/docs/assets/coremeta4cat_vocabulary.xlsx
+++ b/docs/assets/coremeta4cat_vocabulary.xlsx
@@ -21962,7 +21962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -22122,7 +22122,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>catalyst type</t>
+          <t>has catalyst type</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -22138,7 +22138,7 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>CatalystType</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -22161,55 +22161,46 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>reactor temperature range</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr"/>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>QuantitativeRange</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr"/>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>VOC4CAT:0007032</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>Temperature range in the reactor during the reaction, provided as a
-QuantitativeRange with min_value and max_value (unit_code: "Cel").
-For a single set-point, set min_value equal to max_value.</t>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>has catalyst type</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr"/>
+      <c r="F5" s="13" t="inlineStr"/>
+      <c r="G5" s="13" t="inlineStr"/>
+      <c r="H5" s="13" t="inlineStr"/>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007014</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>Type of catalyst used (e.g. heterogeneous, homogeneous, biocatalyst).
+For heterogeneous catalysts, use voc4cat terms where available.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>QuantitativeRange</t>
+          <t>HeterogeneousCatalyst</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
@@ -22219,12 +22210,12 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>reactor temperature range</t>
+          <t>CatalystType</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr"/>
@@ -22233,10 +22224,416 @@
       <c r="H6" s="13" t="inlineStr"/>
       <c r="I6" s="13" t="inlineStr">
         <is>
+          <t>VOC4CAT:0007003</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>A substance that increases the rate of a chemical reaction that is in a different phase than the reagents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>HomogeneousCatalyst</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr"/>
+      <c r="F7" s="13" t="inlineStr"/>
+      <c r="G7" s="13" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>coremeta4cat:HomogeneousCatalyst</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>A substance that increses the rate of a chemical reaction that is in the same phase as the reagents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>BioCatalyst</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr"/>
+      <c r="F8" s="13" t="inlineStr"/>
+      <c r="G8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>coremeta4cat:BioCatalyst</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>An enzyme or cell that catalyzes a biocatalytic reaction. Subclass of Catalyst (AgenticEntity). The physical form in which it is applied is described by an associated BiocatalystPreparation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>ElectroCatalyst</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr"/>
+      <c r="F9" s="13" t="inlineStr"/>
+      <c r="G9" s="13" t="inlineStr"/>
+      <c r="H9" s="13" t="inlineStr"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000255</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>The characteristics of a material or substance that determine how it interacts or responds to a magnetic field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>ThinFilmCatalyst</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000019</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst introduced to the reaction chamber in the form of a thin film. To form a thin film, a (powdered) catalyst is deposited on a substrate (e.g., glass or metal) using an appropriate deposition technique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>BulkCatalyst</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr"/>
+      <c r="F11" s="13" t="inlineStr"/>
+      <c r="G11" s="13" t="inlineStr"/>
+      <c r="H11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007015</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst that consists mainly of the active ingredient or phase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>PowerderedCatalyst</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="13" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr"/>
+      <c r="H12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000017</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst introduced to the reaction chamber in the form of a powder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>DepositedSampleCatalyst</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr"/>
+      <c r="F13" s="13" t="inlineStr"/>
+      <c r="G13" s="13" t="inlineStr"/>
+      <c r="H13" s="13" t="inlineStr"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000038</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>A thin film of the catalyst deposited on an appropriate for the application substrate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>PhotoCatalyst</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr"/>
+      <c r="F14" s="13" t="inlineStr"/>
+      <c r="G14" s="13" t="inlineStr"/>
+      <c r="H14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000002</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>A material that absorbs photons (light) of appropriate energy and initiates or accelerates a photochemical reaction, while it regenerates itself after each reaction cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>SupportedCatalsyt</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>CatalystType</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr"/>
+      <c r="F15" s="13" t="inlineStr"/>
+      <c r="G15" s="13" t="inlineStr"/>
+      <c r="H15" s="13" t="inlineStr"/>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007034</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>A catalyst where the active material is usually the minority phase and fixed on a high surface area, relatively inert solid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>reactor temperature range</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>QuantitativeRange</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr"/>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0007032</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Temperature range in the reactor during the reaction, provided as a
+QuantitativeRange with min_value and max_value (unit_code: "Cel").
+For a single set-point, set min_value equal to max_value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>QuantitativeRange</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>reactor temperature range</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr"/>
+      <c r="F17" s="13" t="inlineStr"/>
+      <c r="G17" s="13" t="inlineStr"/>
+      <c r="H17" s="13" t="inlineStr"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
           <t>qudt:Quantity</t>
         </is>
       </c>
-      <c r="J6" s="13" t="inlineStr">
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>A quantitative property expressed as a range between a lower and upper bound,
 sharing a common unit. Used where an experiment operates over a range of
@@ -22247,271 +22644,271 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr"/>
-      <c r="G7" s="12" t="inlineStr"/>
-      <c r="H7" s="12" t="inlineStr"/>
-      <c r="I7" s="12" t="inlineStr"/>
-      <c r="J7" s="12" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr"/>
+      <c r="G18" s="12" t="inlineStr"/>
+      <c r="H18" s="12" t="inlineStr"/>
+      <c r="I18" s="12" t="inlineStr"/>
+      <c r="J18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr"/>
-      <c r="G8" s="12" t="inlineStr"/>
-      <c r="H8" s="12" t="inlineStr"/>
-      <c r="I8" s="12" t="inlineStr"/>
-      <c r="J8" s="12" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr"/>
+      <c r="G19" s="12" t="inlineStr"/>
+      <c r="H19" s="12" t="inlineStr"/>
+      <c r="I19" s="12" t="inlineStr"/>
+      <c r="J19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>has atmosphere</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr"/>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr"/>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Atmosphere</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr"/>
-      <c r="I9" s="12" t="inlineStr">
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr"/>
+      <c r="I20" s="12" t="inlineStr">
         <is>
           <t>VOC4CAT:0007809</t>
         </is>
       </c>
-      <c r="J9" s="12" t="inlineStr">
+      <c r="J20" s="12" t="inlineStr">
         <is>
           <t>Gaseous environment or atmospheric conditions during a process.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Atmosphere</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>has atmosphere</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr"/>
-      <c r="F10" s="13" t="inlineStr"/>
-      <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr"/>
-      <c r="I10" s="13" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr"/>
+      <c r="F21" s="13" t="inlineStr"/>
+      <c r="G21" s="13" t="inlineStr"/>
+      <c r="H21" s="13" t="inlineStr"/>
+      <c r="I21" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:Atmosphere</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="J21" s="13" t="inlineStr">
         <is>
           <t>A qualitative descriptor of the gaseous environment or atmospheric
 conditions during a process (e.g. "air", "N2", "5% H2/Ar").</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>CalcinationGaseousEnvironment</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>Atmosphere</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr"/>
-      <c r="F11" s="13" t="inlineStr"/>
-      <c r="G11" s="13" t="inlineStr"/>
-      <c r="H11" s="13" t="inlineStr"/>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr"/>
+      <c r="F22" s="13" t="inlineStr"/>
+      <c r="G22" s="13" t="inlineStr"/>
+      <c r="H22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0000055</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J22" s="13" t="inlineStr">
         <is>
           <t>The specific gaseous environment maintained during a calcination step
 (e.g. "air", "N2", "10% O2/N2").</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>experiment pressure</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr"/>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Pressure</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr"/>
-      <c r="I12" s="12" t="inlineStr">
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr"/>
+      <c r="I23" s="12" t="inlineStr">
         <is>
           <t>VOC4CAT:0000118</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr">
+      <c r="J23" s="12" t="inlineStr">
         <is>
           <t>Total pressure in the reactor during the experiment.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>feed composition range</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr"/>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr"/>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="inlineStr"/>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr"/>
+      <c r="I24" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:feed_composition_range</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="J24" s="12" t="inlineStr">
         <is>
           <t>Feed composition range studied, provided as a QuantitativeRange.
 Express concentration bounds in an appropriate unit (e.g. "mol/L", "%" for
@@ -22519,37 +22916,37 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>QuantitativeRange</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>feed composition range</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="inlineStr"/>
-      <c r="F14" s="13" t="inlineStr"/>
-      <c r="G14" s="13" t="inlineStr"/>
-      <c r="H14" s="13" t="inlineStr"/>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr"/>
+      <c r="F25" s="13" t="inlineStr"/>
+      <c r="G25" s="13" t="inlineStr"/>
+      <c r="H25" s="13" t="inlineStr"/>
+      <c r="I25" s="13" t="inlineStr">
         <is>
           <t>qudt:Quantity</t>
         </is>
       </c>
-      <c r="J14" s="13" t="inlineStr">
+      <c r="J25" s="13" t="inlineStr">
         <is>
           <t>A quantitative property expressed as a range between a lower and upper bound,
 sharing a common unit. Used where an experiment operates over a range of
@@ -22560,117 +22957,117 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>has experiment duration</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr"/>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr"/>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr"/>
-      <c r="G15" s="12" t="inlineStr"/>
-      <c r="H15" s="12" t="inlineStr"/>
-      <c r="I15" s="12" t="inlineStr">
+      <c r="F26" s="12" t="inlineStr"/>
+      <c r="G26" s="12" t="inlineStr"/>
+      <c r="H26" s="12" t="inlineStr"/>
+      <c r="I26" s="12" t="inlineStr">
         <is>
           <t>SIO:000008</t>
         </is>
       </c>
-      <c r="J15" s="12" t="inlineStr">
+      <c r="J26" s="12" t="inlineStr">
         <is>
           <t>Total duration of the experiment or measurement run.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>has experiment duration</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr"/>
-      <c r="F16" s="13" t="inlineStr"/>
-      <c r="G16" s="13" t="inlineStr"/>
-      <c r="H16" s="13" t="inlineStr"/>
-      <c r="I16" s="13" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr"/>
+      <c r="F27" s="13" t="inlineStr"/>
+      <c r="G27" s="13" t="inlineStr"/>
+      <c r="H27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0008120</t>
         </is>
       </c>
-      <c r="J16" s="13" t="inlineStr">
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>A quantitative measure of elapsed time (duration of a process step).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>product identification method</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr"/>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr"/>
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>ProductIdentificationMethod</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr"/>
-      <c r="I17" s="11" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr"/>
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>coremeta4cat:product_identification_method</t>
         </is>
       </c>
-      <c r="J17" s="11" t="inlineStr">
+      <c r="J28" s="11" t="inlineStr">
         <is>
           <t>The analytical method used to identify and/or quantify reaction products.
 Should reference a CharacterizationTechnique instance (e.g. GCMS, HPLC_MS).
@@ -22678,37 +23075,37 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>ProductIdentificationMethod</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>product identification method</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr"/>
-      <c r="F18" s="13" t="inlineStr"/>
-      <c r="G18" s="13" t="inlineStr"/>
-      <c r="H18" s="13" t="inlineStr"/>
-      <c r="I18" s="13" t="inlineStr">
+      <c r="E29" s="13" t="inlineStr"/>
+      <c r="F29" s="13" t="inlineStr"/>
+      <c r="G29" s="13" t="inlineStr"/>
+      <c r="H29" s="13" t="inlineStr"/>
+      <c r="I29" s="13" t="inlineStr">
         <is>
           <t>OBI:0000272</t>
         </is>
       </c>
-      <c r="J18" s="13" t="inlineStr">
+      <c r="J29" s="13" t="inlineStr">
         <is>
           <t>Abstract Plan representing the method used to identify and quantify reaction
 products. In practice, users should reference a concrete CharacterizationTechnique
@@ -22719,41 +23116,41 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>carried out by</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr"/>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr"/>
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr"/>
-      <c r="I19" s="11" t="inlineStr"/>
-      <c r="J19" s="11" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr"/>
+      <c r="I30" s="11" t="inlineStr"/>
+      <c r="J30" s="11" t="inlineStr">
         <is>
           <t>The reactor in which the Reaction takes place.
 Must be a Reactor instance (a Device subclass specific to catalytic
@@ -22761,37 +23158,37 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
         <is>
           <t>carried out by</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr"/>
-      <c r="F20" s="13" t="inlineStr"/>
-      <c r="G20" s="13" t="inlineStr"/>
-      <c r="H20" s="13" t="inlineStr"/>
-      <c r="I20" s="13" t="inlineStr">
+      <c r="E31" s="13" t="inlineStr"/>
+      <c r="F31" s="13" t="inlineStr"/>
+      <c r="G31" s="13" t="inlineStr"/>
+      <c r="H31" s="13" t="inlineStr"/>
+      <c r="I31" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0007018</t>
         </is>
       </c>
-      <c r="J20" s="13" t="inlineStr">
+      <c r="J31" s="13" t="inlineStr">
         <is>
           <t>Abstract Device subclass representing a catalytic reactor vessel.
 Reactor is more specific than the general Device (AgenticEntity): it restricts
@@ -22804,222 +23201,222 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>ElectrochemicalReactor</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C32" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D32" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr"/>
-      <c r="F21" s="13" t="inlineStr"/>
-      <c r="G21" s="13" t="inlineStr"/>
-      <c r="H21" s="13" t="inlineStr"/>
-      <c r="I21" s="13" t="inlineStr">
+      <c r="E32" s="13" t="inlineStr"/>
+      <c r="F32" s="13" t="inlineStr"/>
+      <c r="G32" s="13" t="inlineStr"/>
+      <c r="H32" s="13" t="inlineStr"/>
+      <c r="I32" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0000193</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
+      <c r="J32" s="13" t="inlineStr">
         <is>
           <t>Electrochemical reactor used in electrocatalytic experiments, including
 H-cells, flow cells, and membrane electrode assemblies.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>CSTR</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr"/>
-      <c r="F22" s="13" t="inlineStr"/>
-      <c r="G22" s="13" t="inlineStr"/>
-      <c r="H22" s="13" t="inlineStr"/>
-      <c r="I22" s="13" t="inlineStr">
+      <c r="E33" s="13" t="inlineStr"/>
+      <c r="F33" s="13" t="inlineStr"/>
+      <c r="G33" s="13" t="inlineStr"/>
+      <c r="H33" s="13" t="inlineStr"/>
+      <c r="I33" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0007019</t>
         </is>
       </c>
-      <c r="J22" s="13" t="inlineStr">
+      <c r="J33" s="13" t="inlineStr">
         <is>
           <t>Continuous stirred tank reactor (CSTR) — a well-mixed, continuous-flow
 reactor operating at steady state.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>PlugFlowReactor</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C34" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr"/>
-      <c r="F23" s="13" t="inlineStr"/>
-      <c r="G23" s="13" t="inlineStr"/>
-      <c r="H23" s="13" t="inlineStr"/>
-      <c r="I23" s="13" t="inlineStr">
+      <c r="E34" s="13" t="inlineStr"/>
+      <c r="F34" s="13" t="inlineStr"/>
+      <c r="G34" s="13" t="inlineStr"/>
+      <c r="H34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0007102</t>
         </is>
       </c>
-      <c r="J23" s="13" t="inlineStr">
+      <c r="J34" s="13" t="inlineStr">
         <is>
           <t>Plug flow reactor (PFR) — a tubular reactor in which reactant composition
 varies along the axis with no axial mixing.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>Autoclave</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr"/>
-      <c r="F24" s="13" t="inlineStr"/>
-      <c r="G24" s="13" t="inlineStr"/>
-      <c r="H24" s="13" t="inlineStr"/>
-      <c r="I24" s="13" t="inlineStr">
+      <c r="E35" s="13" t="inlineStr"/>
+      <c r="F35" s="13" t="inlineStr"/>
+      <c r="G35" s="13" t="inlineStr"/>
+      <c r="H35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr">
         <is>
           <t>NCIT:C93052</t>
         </is>
       </c>
-      <c r="J24" s="13" t="inlineStr">
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>Autoclave reactor — a sealed pressure vessel for batch reactions at
 elevated temperature and/or pressure.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>SlurryReactor</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C36" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr"/>
-      <c r="F25" s="13" t="inlineStr"/>
-      <c r="G25" s="13" t="inlineStr"/>
-      <c r="H25" s="13" t="inlineStr"/>
-      <c r="I25" s="13" t="inlineStr">
+      <c r="E36" s="13" t="inlineStr"/>
+      <c r="F36" s="13" t="inlineStr"/>
+      <c r="G36" s="13" t="inlineStr"/>
+      <c r="H36" s="13" t="inlineStr"/>
+      <c r="I36" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:SlurryReactor</t>
         </is>
       </c>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="J36" s="13" t="inlineStr">
         <is>
           <t>Slurry reactor — a three-phase reactor in which catalyst particles are
 suspended in a liquid phase through which gas is bubbled.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>Microreactor</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C37" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr"/>
-      <c r="F26" s="13" t="inlineStr"/>
-      <c r="G26" s="13" t="inlineStr"/>
-      <c r="H26" s="13" t="inlineStr"/>
-      <c r="I26" s="13" t="inlineStr">
+      <c r="E37" s="13" t="inlineStr"/>
+      <c r="F37" s="13" t="inlineStr"/>
+      <c r="G37" s="13" t="inlineStr"/>
+      <c r="H37" s="13" t="inlineStr"/>
+      <c r="I37" s="13" t="inlineStr">
         <is>
           <t>VOC4CAT:0000234</t>
         </is>
       </c>
-      <c r="J26" s="13" t="inlineStr">
+      <c r="J37" s="13" t="inlineStr">
         <is>
           <t>Microreactor — a miniaturised flow reactor with characteristic dimensions
 in the sub-millimetre range, enabling precise thermal control and rapid
@@ -23027,207 +23424,207 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>FixedBedReactor</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C38" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr"/>
-      <c r="F27" s="13" t="inlineStr"/>
-      <c r="G27" s="13" t="inlineStr"/>
-      <c r="H27" s="13" t="inlineStr"/>
-      <c r="I27" s="13" t="inlineStr">
+      <c r="E38" s="13" t="inlineStr"/>
+      <c r="F38" s="13" t="inlineStr"/>
+      <c r="G38" s="13" t="inlineStr"/>
+      <c r="H38" s="13" t="inlineStr"/>
+      <c r="I38" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:FixedBedReactor</t>
         </is>
       </c>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="J38" s="13" t="inlineStr">
         <is>
           <t>Fixed bed reactor — a tubular reactor packed with a stationary catalyst bed.
 The most common reactor type in heterogeneous catalysis testing.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr"/>
-      <c r="F28" s="13" t="inlineStr"/>
-      <c r="G28" s="13" t="inlineStr"/>
-      <c r="H28" s="13" t="inlineStr"/>
-      <c r="I28" s="13" t="inlineStr">
+      <c r="E39" s="13" t="inlineStr"/>
+      <c r="F39" s="13" t="inlineStr"/>
+      <c r="G39" s="13" t="inlineStr"/>
+      <c r="H39" s="13" t="inlineStr"/>
+      <c r="I39" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="J28" s="13" t="inlineStr">
+      <c r="J39" s="13" t="inlineStr">
         <is>
           <t>Fluidized bed reactor — a reactor in which the catalyst particles are
 suspended in an upward-flowing gas or liquid stream.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>gas distributor type</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G29" s="12" t="inlineStr"/>
-      <c r="H29" s="12" t="inlineStr"/>
-      <c r="I29" s="12" t="inlineStr">
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr"/>
+      <c r="H40" s="12" t="inlineStr"/>
+      <c r="I40" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:gas_distributor_type</t>
         </is>
       </c>
-      <c r="J29" s="12" t="inlineStr">
+      <c r="J40" s="12" t="inlineStr">
         <is>
           <t>Type or design of the gas distributor plate in a fluidized bed reactor.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>bed expansion height</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="inlineStr"/>
-      <c r="H30" s="12" t="inlineStr">
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr"/>
+      <c r="H41" s="12" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="I30" s="12" t="inlineStr">
+      <c r="I41" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:bed_expansion_height</t>
         </is>
       </c>
-      <c r="J30" s="12" t="inlineStr">
+      <c r="J41" s="12" t="inlineStr">
         <is>
           <t>Height of bed expansion above the settled bed height under operating conditions.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>bubble size distribution</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr"/>
-      <c r="G31" s="12" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr"/>
-      <c r="I31" s="12" t="inlineStr">
+      <c r="F42" s="12" t="inlineStr"/>
+      <c r="G42" s="12" t="inlineStr"/>
+      <c r="H42" s="12" t="inlineStr"/>
+      <c r="I42" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:bubble_size_distribution</t>
         </is>
       </c>
-      <c r="J31" s="12" t="inlineStr">
+      <c r="J42" s="12" t="inlineStr">
         <is>
           <t>Description or characterization of bubble size distribution in the fluidized bed.</t>
         </is>

</xml_diff>

<commit_message>
update CatalyticReaction test data
</commit_message>
<xml_diff>
--- a/docs/assets/coremeta4cat_vocabulary.xlsx
+++ b/docs/assets/coremeta4cat_vocabulary.xlsx
@@ -22562,40 +22562,40 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>has reaction type</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr"/>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr"/>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>ReactionType</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr"/>
-      <c r="H16" s="11" t="inlineStr"/>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr"/>
+      <c r="H16" s="10" t="inlineStr"/>
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>VOC4CAT:0007010</t>
         </is>
       </c>
-      <c r="J16" s="11" t="inlineStr">
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>A group of chemical reactions with common conditions or reactants, e.g. Oxidation, Hydrogenation, Reduction, Cracking.</t>
         </is>
@@ -22619,7 +22619,7 @@
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr"/>
@@ -22655,7 +22655,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr"/>
@@ -22676,7 +22676,7 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>CO2-Hydrogenation</t>
+          <t>CarbonDioxideHydrogenation</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -22691,7 +22691,7 @@
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr"/>
@@ -22727,7 +22727,7 @@
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr"/>
@@ -22763,7 +22763,7 @@
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr"/>
@@ -22784,7 +22784,7 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>CO-Oxidation</t>
+          <t>CarbonMonoxideOxidation</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
@@ -22799,7 +22799,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr"/>
@@ -22835,7 +22835,7 @@
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr"/>
@@ -22856,7 +22856,7 @@
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>C-C-CouplingReaction</t>
+          <t>CarbonCouplingReaction</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
@@ -22871,7 +22871,7 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr"/>
@@ -22907,7 +22907,7 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr"/>
@@ -22943,7 +22943,7 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr"/>
@@ -22979,7 +22979,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr"/>
@@ -23015,7 +23015,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>R</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr"/>
@@ -24681,7 +24681,7 @@
       <c r="H70" s="13" t="inlineStr"/>
       <c r="I70" s="13" t="inlineStr">
         <is>
-          <t>VOc4CAT:0007813</t>
+          <t>VOC4CAT:0007813</t>
         </is>
       </c>
       <c r="J70" s="13" t="inlineStr">

</xml_diff>